<commit_message>
add sourcegrid column to hp-input. remove debug printing.
</commit_message>
<xml_diff>
--- a/example_data/production/hp-input.xlsx
+++ b/example_data/production/hp-input.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
   <si>
     <t xml:space="preserve">block_identifier</t>
   </si>
@@ -32,6 +32,9 @@
     <t xml:space="preserve">type</t>
   </si>
   <si>
+    <t xml:space="preserve">sourcegrid</t>
+  </si>
+  <si>
     <t xml:space="preserve">unit_capacity</t>
   </si>
   <si>
@@ -62,9 +65,6 @@
     <t xml:space="preserve">co2</t>
   </si>
   <si>
-    <t xml:space="preserve">Explanation of the data columns in Sheet1:</t>
-  </si>
-  <si>
     <t xml:space="preserve">column</t>
   </si>
   <si>
@@ -77,7 +77,10 @@
     <t xml:space="preserve">name of the city block where the production unit lies</t>
   </si>
   <si>
-    <t xml:space="preserve">“heat” for heating heat pumps or “cool”</t>
+    <t xml:space="preserve">States the output grid.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">States the grid of the source energy.</t>
   </si>
   <si>
     <t xml:space="preserve">Alternative which the given values are for</t>
@@ -211,7 +214,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -226,10 +229,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -427,17 +426,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="16.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="24.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="16.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="15.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="21.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15.07"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -471,36 +470,40 @@
       <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="F2" s="1" t="n">
         <v>60000</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="G2" s="1" t="n">
         <v>0.98</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="H2" s="1" t="n">
         <v>1000</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="1" t="n">
+      <c r="I2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="1" t="n">
         <v>0.002</v>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="K2" s="1" t="n">
         <v>150</v>
       </c>
     </row>
@@ -508,264 +511,317 @@
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
+      <c r="D54" s="3"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -783,7 +839,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.36"/>
@@ -792,118 +848,122 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>13</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>16</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>0</v>
+      <c r="A4" s="5" t="s">
+        <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="6"/>
+        <v>19</v>
+      </c>
+      <c r="C4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="6"/>
+      <c r="A5" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>1</v>
+      <c r="A6" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="6"/>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="7" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="7" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="23.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="C7" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="6"/>
+    </row>
+    <row r="9" customFormat="false" ht="46.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="7"/>
-    </row>
-    <row r="10" customFormat="false" ht="46.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="7"/>
-    </row>
-    <row r="12" customFormat="false" ht="34.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="23.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C10" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="34.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="7" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="23.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>31</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
small correction to example data.
</commit_message>
<xml_diff>
--- a/example_data/production/hp-input.xlsx
+++ b/example_data/production/hp-input.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
@@ -426,7 +426,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.93"/>
@@ -506,322 +506,6 @@
       <c r="K2" s="1" t="n">
         <v>150</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-    </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-    </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-    </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-    </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
-    </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-    </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-    </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-    </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3"/>
-      <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-    </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-    </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-    </row>
-    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-    </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
-      <c r="D49" s="3"/>
-    </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-    </row>
-    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="3"/>
-      <c r="D51" s="3"/>
-    </row>
-    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3"/>
-      <c r="B52" s="3"/>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-    </row>
-    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3"/>
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
-    </row>
-    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-    </row>
-    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3"/>
-      <c r="B55" s="3"/>
-      <c r="C55" s="3"/>
-      <c r="D55" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>